<commit_message>
Orden y actualización de los datos
</commit_message>
<xml_diff>
--- a/input/Clasificacion.xlsx
+++ b/input/Clasificacion.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soledadaraya/Library/CloudStorage/Dropbox/Lucía Miranda Fondecyt/femocratas/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DD13220-C50B-6146-88F6-C2FB43C6BCFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BEAD3C-01BC-4E40-B9F1-FE50B318DF2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$F$44</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="48">
   <si>
     <t>Entrevistas</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t>Chile</t>
+  </si>
+  <si>
+    <t>Estado-Punto focal</t>
   </si>
 </sst>
 </file>
@@ -495,13 +498,13 @@
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>7</v>
@@ -510,12 +513,12 @@
         <v>8</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>44</v>
@@ -535,7 +538,7 @@
     </row>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>44</v>
@@ -555,13 +558,13 @@
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>7</v>
@@ -570,84 +573,92 @@
         <v>8</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="4"/>
+        <v>29</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>44</v>
@@ -667,16 +678,16 @@
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
@@ -687,7 +698,7 @@
     </row>
     <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>44</v>
@@ -699,15 +710,15 @@
         <v>7</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>44</v>
@@ -727,13 +738,13 @@
     </row>
     <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>7</v>
@@ -747,7 +758,7 @@
     </row>
     <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>44</v>
@@ -759,21 +770,21 @@
         <v>7</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>7</v>
@@ -782,12 +793,12 @@
         <v>8</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>44</v>
@@ -802,36 +813,38 @@
         <v>8</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F18" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>7</v>
@@ -840,18 +853,18 @@
         <v>8</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>7</v>
@@ -860,173 +873,123 @@
         <v>8</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3" t="s">
-        <v>36</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>9</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>9</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>36</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>36</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1034,67 +997,55 @@
         <v>21</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>9</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F32" s="4"/>
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>38</v>
+      <c r="C33" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>36</v>
@@ -1103,148 +1054,202 @@
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>9</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F34" s="4"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="F35" s="4"/>
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F36" s="4"/>
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="F38" s="4"/>
     </row>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="F39" s="4"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F40" s="4"/>
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F41" s="4"/>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F42" s="4"/>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F43" s="4"/>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+        <v>45</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="F44" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F44">
-      <sortCondition ref="D1:D44"/>
+  <autoFilter ref="A1:F44" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F21">
+      <sortCondition ref="A1:A44"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>